<commit_message>
feat(shortcycle): integrate accepted layout and workflow stage
Finalize accepted visibility timing, tray transitions, modal anchors and localized cover bubbles.
Include the repaired authoring workbook, configuration guide, current layout inputs and bounded workflow continuation.
Preserve stage records while excluding local review exports and dynamic font runtime cache.

Validation: ShortCycle compilation/behavior checks pass (94 inputs, 282 static assertions); 16 Workflow runners pass.
Legacy documentation index checks remain reported in the stage review; no test threshold or historical ledger content was changed.
</commit_message>
<xml_diff>
--- a/DevTools/DataTables/Authoring/DataTables_Authoring.xlsx
+++ b/DevTools/DataTables/Authoring/DataTables_Authoring.xlsx
@@ -5044,9 +5044,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.########"/>
     <numFmt numFmtId="165" formatCode="0.########"/>
+    <numFmt numFmtId="166" formatCode="0.########"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -5192,7 +5193,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -5243,6 +5244,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -9710,10 +9720,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0900-000000000000}">
@@ -9950,10 +9956,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0A00-000000000000}">
@@ -10376,10 +10378,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0B00-000001000000}">
@@ -10785,10 +10783,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0C00-000001000000}">
@@ -10814,7 +10808,7 @@
   <sheetPr>
     <tabColor rgb="FF7E57C2"/>
   </sheetPr>
-  <dimension ref="A1:K158"/>
+  <dimension ref="A1:K160"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -12339,6 +12333,30 @@
       </c>
       <c r="B158" s="9" t="s">
         <v>862</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t>ui_p0_cover_bubble_a.text</t>
+        </is>
+      </c>
+      <c r="B159" s="1" t="inlineStr">
+        <is>
+          <t>吃什么</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" spans="1:3">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t>ui_p0_cover_bubble_b.text</t>
+        </is>
+      </c>
+      <c r="B160" s="1" t="inlineStr">
+        <is>
+          <t>汪！</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -12474,7 +12492,6 @@
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
-  <dataValidations count="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -12647,10 +12664,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0200-000000000000}">
@@ -13955,10 +13968,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000002000000}">
@@ -14221,10 +14230,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0400-000001000000}">
@@ -14458,10 +14463,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0500-000001000000}">
@@ -15404,10 +15405,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0700-000002000000}">
@@ -15857,10 +15854,6 @@
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-      </x14:conditionalFormattings>
-    </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0800-000001000000}">

</xml_diff>